<commit_message>
Updated requirements_traceability.xlsx for sprint 1
</commit_message>
<xml_diff>
--- a/Evidence/REQM/requirements_traceability.xlsx
+++ b/Evidence/REQM/requirements_traceability.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095-Group-16-Music-Player-Application\Evidence\REQM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8EE13C5-217C-462A-89F6-6C0671A52E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF5370F0-C61D-4CFC-8141-F3E033286837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{69E9F38F-E908-4412-9BBE-056D5BFD6B03}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="191">
   <si>
     <t>Story ID</t>
   </si>
@@ -510,13 +510,112 @@
   </si>
   <si>
     <t>Backlog</t>
+  </si>
+  <si>
+    <t>player_core.py, player_state.py</t>
+  </si>
+  <si>
+    <t>player_queue.py</t>
+  </si>
+  <si>
+    <t>player_ui</t>
+  </si>
+  <si>
+    <t>player_audio.py</t>
+  </si>
+  <si>
+    <t>player_seek.py</t>
+  </si>
+  <si>
+    <t>player_ui.py</t>
+  </si>
+  <si>
+    <t>player_shortcuts.py</t>
+  </si>
+  <si>
+    <t>player_help.py</t>
+  </si>
+  <si>
+    <t>player_core.py</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-11-help-commands</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-06-progress-bar-and-time-skipping</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-09-mute-unmute</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-05-song-progress-total-time-spent</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-04-volume</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-08-rewind-and-fast-forward</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-07-keyboard-shortcuts</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-10-song-indicator</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-03-song-info</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-02-next-previous</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-12-background-music</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S1-01-play-pause</t>
+  </si>
+  <si>
+    <t>test_music_player_player_core.py, test_music_player_player_state.py, ra495_blackbox_specification_test.py, extra_test.py, player_core_branch_test.py, player_core_statement_test.py, player_state_branch_test.py, player_state_statement_test.py</t>
+  </si>
+  <si>
+    <t>sp871_specification_test.py, test_music_player_player_queue.py, player_queue_branch_test.py, player_queue_statement_test.py</t>
+  </si>
+  <si>
+    <t>ra495_blackbox_specification_test.py, ra495_player_ui_branch_test.py, ra495_player_ui_statement_test.py</t>
+  </si>
+  <si>
+    <t>test_music_player_player_audio.py, sa1077_player_audio_branch_test.py, sa1077_player_audio_statement_test.py, sa1077_specification_test.py</t>
+  </si>
+  <si>
+    <t>sa1077_specification_test.py, sa1077_player_ui_branch_test.py, sa1077_player_ui_statement_test.py</t>
+  </si>
+  <si>
+    <t>sa1077_specification_test.py, player_seek_branch_test.py, player_seek_statement_test.py, test_music_player_player_seek.py, test_music_player_time_utils.py, time_utils_branch_test.py, time_utils_statement_test.py</t>
+  </si>
+  <si>
+    <t>np343_blackbox_specification_test.py, player_shortcuts_branch_test.py, player_shortcuts_statement_test.py, test_music_player_player_shortcuts.py</t>
+  </si>
+  <si>
+    <t>np343_blackbox_specification_test.py, test_music_player_player_seek.py, sa1077_specification_test.py, player_seek_branch_test.py, player_seek_statement_test.py</t>
+  </si>
+  <si>
+    <t>sp871_specification_test.py, sp871_player_audio_branch_test.py, sp871_player_audio_statement_test.py</t>
+  </si>
+  <si>
+    <t>ra495_blackbox_specification_test.py, ra495_player_ui_branch_test.py, ra495_player_ui_statement_test.py, test_music_player_player_ui.py</t>
+  </si>
+  <si>
+    <t>test_music_player_player_help.py, sp871_specification_test.py, player_help_branch_test.py, player_help_statement_test.py</t>
+  </si>
+  <si>
+    <t>test_music_player_player_core.py, ra495_blackbox_specification_test.py, player_core_branch_test.py, player_core_statement_test.py, extra_test.py</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -534,6 +633,14 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -556,18 +663,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -907,11 +1017,11 @@
     <col min="3" max="3" width="6.85546875" customWidth="1"/>
     <col min="4" max="4" width="19.28515625" customWidth="1"/>
     <col min="5" max="5" width="88.42578125" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" customWidth="1"/>
-    <col min="7" max="7" width="16.42578125" customWidth="1"/>
+    <col min="6" max="6" width="29.42578125" customWidth="1"/>
+    <col min="7" max="7" width="215.85546875" customWidth="1"/>
     <col min="8" max="8" width="12.5703125" customWidth="1"/>
     <col min="9" max="9" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="21.42578125" customWidth="1"/>
+    <col min="10" max="10" width="118.5703125" customWidth="1"/>
     <col min="11" max="11" width="13.140625" customWidth="1"/>
     <col min="12" max="12" width="14.140625" customWidth="1"/>
   </cols>
@@ -968,11 +1078,23 @@
       <c r="E2" t="s">
         <v>109</v>
       </c>
+      <c r="F2" t="s">
+        <v>158</v>
+      </c>
+      <c r="G2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H2">
+        <v>100</v>
+      </c>
       <c r="I2" t="s">
         <v>157</v>
       </c>
+      <c r="J2" s="4" t="s">
+        <v>178</v>
+      </c>
       <c r="K2" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -991,11 +1113,23 @@
       <c r="E3" t="s">
         <v>110</v>
       </c>
+      <c r="F3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G3" t="s">
+        <v>180</v>
+      </c>
+      <c r="H3">
+        <v>75</v>
+      </c>
       <c r="I3" t="s">
         <v>157</v>
       </c>
+      <c r="J3" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="K3" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1014,11 +1148,23 @@
       <c r="E4" t="s">
         <v>111</v>
       </c>
+      <c r="F4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G4" t="s">
+        <v>181</v>
+      </c>
+      <c r="H4">
+        <v>100</v>
+      </c>
       <c r="I4" t="s">
         <v>157</v>
       </c>
+      <c r="J4" s="4" t="s">
+        <v>175</v>
+      </c>
       <c r="K4" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -1037,11 +1183,23 @@
       <c r="E5" t="s">
         <v>150</v>
       </c>
+      <c r="F5" t="s">
+        <v>161</v>
+      </c>
+      <c r="G5" t="s">
+        <v>182</v>
+      </c>
+      <c r="H5">
+        <v>100</v>
+      </c>
       <c r="I5" t="s">
         <v>157</v>
       </c>
+      <c r="J5" s="4" t="s">
+        <v>171</v>
+      </c>
       <c r="K5" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1060,11 +1218,23 @@
       <c r="E6" t="s">
         <v>112</v>
       </c>
+      <c r="F6" t="s">
+        <v>163</v>
+      </c>
+      <c r="G6" t="s">
+        <v>183</v>
+      </c>
+      <c r="H6">
+        <v>100</v>
+      </c>
       <c r="I6" t="s">
         <v>157</v>
       </c>
+      <c r="J6" s="4" t="s">
+        <v>170</v>
+      </c>
       <c r="K6" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1083,11 +1253,23 @@
       <c r="E7" t="s">
         <v>113</v>
       </c>
+      <c r="F7" t="s">
+        <v>162</v>
+      </c>
+      <c r="G7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H7">
+        <v>100</v>
+      </c>
       <c r="I7" t="s">
         <v>157</v>
       </c>
+      <c r="J7" s="4" t="s">
+        <v>168</v>
+      </c>
       <c r="K7" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -1106,11 +1288,23 @@
       <c r="E8" t="s">
         <v>114</v>
       </c>
+      <c r="F8" t="s">
+        <v>164</v>
+      </c>
+      <c r="G8" t="s">
+        <v>185</v>
+      </c>
+      <c r="H8">
+        <v>100</v>
+      </c>
       <c r="I8" t="s">
         <v>157</v>
       </c>
+      <c r="J8" s="4" t="s">
+        <v>173</v>
+      </c>
       <c r="K8" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1129,11 +1323,23 @@
       <c r="E9" t="s">
         <v>115</v>
       </c>
+      <c r="F9" t="s">
+        <v>162</v>
+      </c>
+      <c r="G9" t="s">
+        <v>186</v>
+      </c>
+      <c r="H9">
+        <v>100</v>
+      </c>
       <c r="I9" t="s">
         <v>157</v>
       </c>
+      <c r="J9" s="4" t="s">
+        <v>172</v>
+      </c>
       <c r="K9" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -1152,11 +1358,23 @@
       <c r="E10" t="s">
         <v>116</v>
       </c>
+      <c r="F10" t="s">
+        <v>161</v>
+      </c>
+      <c r="G10" t="s">
+        <v>187</v>
+      </c>
+      <c r="H10">
+        <v>100</v>
+      </c>
       <c r="I10" t="s">
         <v>157</v>
       </c>
+      <c r="J10" s="4" t="s">
+        <v>169</v>
+      </c>
       <c r="K10" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -1175,11 +1393,23 @@
       <c r="E11" t="s">
         <v>117</v>
       </c>
+      <c r="F11" t="s">
+        <v>163</v>
+      </c>
+      <c r="G11" t="s">
+        <v>188</v>
+      </c>
+      <c r="H11">
+        <v>93</v>
+      </c>
       <c r="I11" t="s">
         <v>157</v>
       </c>
+      <c r="J11" s="4" t="s">
+        <v>174</v>
+      </c>
       <c r="K11" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -1198,11 +1428,23 @@
       <c r="E12" t="s">
         <v>118</v>
       </c>
+      <c r="F12" t="s">
+        <v>165</v>
+      </c>
+      <c r="G12" t="s">
+        <v>189</v>
+      </c>
+      <c r="H12">
+        <v>100</v>
+      </c>
       <c r="I12" t="s">
         <v>157</v>
       </c>
+      <c r="J12" s="4" t="s">
+        <v>167</v>
+      </c>
       <c r="K12" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -1221,11 +1463,23 @@
       <c r="E13" t="s">
         <v>119</v>
       </c>
+      <c r="F13" t="s">
+        <v>166</v>
+      </c>
+      <c r="G13" t="s">
+        <v>190</v>
+      </c>
+      <c r="H13">
+        <v>100</v>
+      </c>
       <c r="I13" t="s">
         <v>157</v>
       </c>
+      <c r="J13" s="4" t="s">
+        <v>177</v>
+      </c>
       <c r="K13" s="3">
-        <v>45973</v>
+        <v>45993</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -2057,6 +2311,20 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J12" r:id="rId1" xr:uid="{3F8D44C8-F061-4367-B70C-9D38E43EEBF7}"/>
+    <hyperlink ref="J7" r:id="rId2" xr:uid="{07BB3D38-21FE-48F7-BA31-D9360AC2C1B2}"/>
+    <hyperlink ref="J10" r:id="rId3" xr:uid="{98B5085D-BC3C-4BA5-8B6A-C6640DAAE840}"/>
+    <hyperlink ref="J6" r:id="rId4" xr:uid="{345855EB-85A7-432D-B808-7548D6CED3EC}"/>
+    <hyperlink ref="J5" r:id="rId5" xr:uid="{CE4744A3-7888-4906-B759-E25B3A066C41}"/>
+    <hyperlink ref="J9" r:id="rId6" xr:uid="{A4A738A8-5311-405A-AB9A-699DDFE42174}"/>
+    <hyperlink ref="J8" r:id="rId7" xr:uid="{426ED8E3-B37E-40E8-9A3B-ABA8F1ABD897}"/>
+    <hyperlink ref="J11" r:id="rId8" xr:uid="{E6BF8555-C0F9-42F4-9D5F-9027F3F5FB4D}"/>
+    <hyperlink ref="J4" r:id="rId9" xr:uid="{75425B77-CF9D-4BC4-B354-1DED57CE5F7B}"/>
+    <hyperlink ref="J3" r:id="rId10" xr:uid="{642AF2ED-DF1B-4C99-811E-B1950408D11F}"/>
+    <hyperlink ref="J13" r:id="rId11" xr:uid="{CE31A3EA-CA0D-4D7A-AA8D-0BFCA3CB5A8A}"/>
+    <hyperlink ref="J2" r:id="rId12" xr:uid="{4B055461-9FA0-4B2F-AD8C-991B813205C3}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated requirements_traceability.xlsx for Sprint 2
</commit_message>
<xml_diff>
--- a/Evidence/REQM/requirements_traceability.xlsx
+++ b/Evidence/REQM/requirements_traceability.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095-Group-16-Music-Player-Application\Evidence\REQM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095\Evidence\REQM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF5370F0-C61D-4CFC-8141-F3E033286837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA06A936-E665-4354-8B47-D826D6D9F425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{69E9F38F-E908-4412-9BBE-056D5BFD6B03}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="16186" xr2:uid="{69E9F38F-E908-4412-9BBE-056D5BFD6B03}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="214">
   <si>
     <t>Story ID</t>
   </si>
@@ -609,6 +609,75 @@
   </si>
   <si>
     <t>test_music_player_player_core.py, ra495_blackbox_specification_test.py, player_core_branch_test.py, player_core_statement_test.py, extra_test.py</t>
+  </si>
+  <si>
+    <t>playlist_model.py, playlists_basic.py</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-01-create-playlist</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-02-add-remove-change-songs</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-03-Search-Song</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-04-View-Songs-Albums-Artists</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-05-playlist-lists</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-06-playlist-contents-autoplay</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-07-add-songs</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-08-confirmation-message</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-09-scan-folder</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-10-number-of-songs-and-total-playtime</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-11-merge-two-playlists-and-remove-duplicate-songs</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S2-12-copy-of-playlist</t>
+  </si>
+  <si>
+    <t>playlists_edit.py</t>
+  </si>
+  <si>
+    <t>library_search_scan.py</t>
+  </si>
+  <si>
+    <t>playlists_basic.py</t>
+  </si>
+  <si>
+    <t>playlists_advanced.py</t>
+  </si>
+  <si>
+    <t>test_music_player_playlist_model.py, test_music_player_playlists_basic.py, test_bb_playlist_model.py, test_bb_playlists_basic.py, test_whitebox_playlist_model_branch.py, test_whitebox_playlist_model_statement.py, test_whitebox_playlists_basic_branch.py, test_whitebox_playlists_basic_statement.py</t>
+  </si>
+  <si>
+    <t>test_music_player_playlists_basic.py, test_bb_playlists_basic.py, test_whitebox_playlists_basic_branch.py, test_whitebox_playlists_basic_statement.py</t>
+  </si>
+  <si>
+    <t>test_music_player_playlists_edit.py, test_sp871_playlists_edit_specification.py, tests_playlists_edit_branch.py, tests_playlists_edit_statement.py</t>
+  </si>
+  <si>
+    <t>test_blackbox_library_search_scan.py, test_music_player_library_search_scan.py, test_whitebox_library_search_scan_branch.py, test_whitebox_library_search_scan_statement.py</t>
+  </si>
+  <si>
+    <t>test_music_player_playlists_advanced.py, test_np343_blackbox_specification_playlists_advanced.py, test_whitebox_playlists_advanced_branch.py, test_whitebox_playlists_advanced_statement.py</t>
   </si>
 </sst>
 </file>
@@ -1011,22 +1080,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C023A292-D7D7-42AA-A66D-EAC889642A87}">
   <dimension ref="A1:L49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="2" max="2" width="146.85546875" customWidth="1"/>
-    <col min="3" max="3" width="6.85546875" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" customWidth="1"/>
-    <col min="5" max="5" width="88.42578125" customWidth="1"/>
-    <col min="6" max="6" width="29.42578125" customWidth="1"/>
-    <col min="7" max="7" width="215.85546875" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="118.5703125" customWidth="1"/>
-    <col min="11" max="11" width="13.140625" customWidth="1"/>
-    <col min="12" max="12" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="146.87890625" customWidth="1"/>
+    <col min="3" max="3" width="6.87890625" customWidth="1"/>
+    <col min="4" max="4" width="19.29296875" customWidth="1"/>
+    <col min="5" max="5" width="88.41015625" customWidth="1"/>
+    <col min="6" max="6" width="29.41015625" customWidth="1"/>
+    <col min="7" max="7" width="236.29296875" customWidth="1"/>
+    <col min="8" max="8" width="12.5859375" customWidth="1"/>
+    <col min="9" max="9" width="12.703125" customWidth="1"/>
+    <col min="10" max="10" width="118.5859375" customWidth="1"/>
+    <col min="11" max="11" width="13.1171875" customWidth="1"/>
+    <col min="12" max="12" width="14.1171875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1062,7 +1131,7 @@
       </c>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>50</v>
       </c>
@@ -1088,7 +1157,7 @@
         <v>100</v>
       </c>
       <c r="I2" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J2" s="4" t="s">
         <v>178</v>
@@ -1097,7 +1166,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
         <v>51</v>
       </c>
@@ -1123,7 +1192,7 @@
         <v>75</v>
       </c>
       <c r="I3" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J3" s="4" t="s">
         <v>176</v>
@@ -1132,7 +1201,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -1158,7 +1227,7 @@
         <v>100</v>
       </c>
       <c r="I4" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>175</v>
@@ -1167,7 +1236,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -1193,7 +1262,7 @@
         <v>100</v>
       </c>
       <c r="I5" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J5" s="4" t="s">
         <v>171</v>
@@ -1202,7 +1271,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -1228,7 +1297,7 @@
         <v>100</v>
       </c>
       <c r="I6" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J6" s="4" t="s">
         <v>170</v>
@@ -1237,7 +1306,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -1263,7 +1332,7 @@
         <v>100</v>
       </c>
       <c r="I7" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J7" s="4" t="s">
         <v>168</v>
@@ -1272,7 +1341,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
         <v>55</v>
       </c>
@@ -1298,7 +1367,7 @@
         <v>100</v>
       </c>
       <c r="I8" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J8" s="4" t="s">
         <v>173</v>
@@ -1307,7 +1376,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -1333,7 +1402,7 @@
         <v>100</v>
       </c>
       <c r="I9" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J9" s="4" t="s">
         <v>172</v>
@@ -1342,7 +1411,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
         <v>57</v>
       </c>
@@ -1368,7 +1437,7 @@
         <v>100</v>
       </c>
       <c r="I10" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J10" s="4" t="s">
         <v>169</v>
@@ -1377,7 +1446,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -1403,7 +1472,7 @@
         <v>93</v>
       </c>
       <c r="I11" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J11" s="4" t="s">
         <v>174</v>
@@ -1412,7 +1481,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -1438,7 +1507,7 @@
         <v>100</v>
       </c>
       <c r="I12" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J12" s="4" t="s">
         <v>167</v>
@@ -1447,7 +1516,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
         <v>60</v>
       </c>
@@ -1473,7 +1542,7 @@
         <v>100</v>
       </c>
       <c r="I13" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="J13" s="4" t="s">
         <v>177</v>
@@ -1482,7 +1551,7 @@
         <v>45993</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A14" t="s">
         <v>62</v>
       </c>
@@ -1498,14 +1567,26 @@
       <c r="E14" t="s">
         <v>120</v>
       </c>
+      <c r="F14" t="s">
+        <v>191</v>
+      </c>
+      <c r="G14" t="s">
+        <v>209</v>
+      </c>
+      <c r="H14">
+        <v>89</v>
+      </c>
       <c r="I14" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>193</v>
       </c>
       <c r="K14" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
         <v>63</v>
       </c>
@@ -1521,14 +1602,26 @@
       <c r="E15" t="s">
         <v>121</v>
       </c>
+      <c r="F15" t="s">
+        <v>205</v>
+      </c>
+      <c r="G15" t="s">
+        <v>211</v>
+      </c>
+      <c r="H15">
+        <v>99</v>
+      </c>
       <c r="I15" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>194</v>
       </c>
       <c r="K15" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
         <v>64</v>
       </c>
@@ -1544,14 +1637,26 @@
       <c r="E16" t="s">
         <v>122</v>
       </c>
+      <c r="F16" t="s">
+        <v>206</v>
+      </c>
+      <c r="G16" t="s">
+        <v>212</v>
+      </c>
+      <c r="H16">
+        <v>97</v>
+      </c>
       <c r="I16" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="K16" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A17" t="s">
         <v>65</v>
       </c>
@@ -1567,14 +1672,26 @@
       <c r="E17" t="s">
         <v>123</v>
       </c>
+      <c r="F17" t="s">
+        <v>206</v>
+      </c>
+      <c r="G17" t="s">
+        <v>212</v>
+      </c>
+      <c r="H17">
+        <v>97</v>
+      </c>
       <c r="I17" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>196</v>
       </c>
       <c r="K17" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A18" t="s">
         <v>66</v>
       </c>
@@ -1590,14 +1707,26 @@
       <c r="E18" t="s">
         <v>124</v>
       </c>
+      <c r="F18" t="s">
+        <v>207</v>
+      </c>
+      <c r="G18" t="s">
+        <v>210</v>
+      </c>
+      <c r="H18">
+        <v>89</v>
+      </c>
       <c r="I18" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>197</v>
       </c>
       <c r="K18" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A19" t="s">
         <v>67</v>
       </c>
@@ -1613,14 +1742,26 @@
       <c r="E19" t="s">
         <v>125</v>
       </c>
+      <c r="F19" t="s">
+        <v>207</v>
+      </c>
+      <c r="G19" t="s">
+        <v>210</v>
+      </c>
+      <c r="H19">
+        <v>89</v>
+      </c>
       <c r="I19" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>198</v>
       </c>
       <c r="K19" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A20" t="s">
         <v>68</v>
       </c>
@@ -1636,14 +1777,26 @@
       <c r="E20" t="s">
         <v>126</v>
       </c>
+      <c r="F20" t="s">
+        <v>205</v>
+      </c>
+      <c r="G20" t="s">
+        <v>211</v>
+      </c>
+      <c r="H20">
+        <v>99</v>
+      </c>
       <c r="I20" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>199</v>
       </c>
       <c r="K20" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A21" t="s">
         <v>69</v>
       </c>
@@ -1659,14 +1812,26 @@
       <c r="E21" t="s">
         <v>127</v>
       </c>
+      <c r="F21" t="s">
+        <v>205</v>
+      </c>
+      <c r="G21" t="s">
+        <v>211</v>
+      </c>
+      <c r="H21">
+        <v>99</v>
+      </c>
       <c r="I21" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>200</v>
       </c>
       <c r="K21" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A22" t="s">
         <v>70</v>
       </c>
@@ -1682,14 +1847,26 @@
       <c r="E22" t="s">
         <v>128</v>
       </c>
+      <c r="F22" t="s">
+        <v>206</v>
+      </c>
+      <c r="G22" t="s">
+        <v>212</v>
+      </c>
+      <c r="H22">
+        <v>97</v>
+      </c>
       <c r="I22" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>201</v>
       </c>
       <c r="K22" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A23" t="s">
         <v>71</v>
       </c>
@@ -1705,14 +1882,26 @@
       <c r="E23" t="s">
         <v>129</v>
       </c>
+      <c r="F23" t="s">
+        <v>207</v>
+      </c>
+      <c r="G23" t="s">
+        <v>210</v>
+      </c>
+      <c r="H23">
+        <v>89</v>
+      </c>
       <c r="I23" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>202</v>
       </c>
       <c r="K23" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A24" t="s">
         <v>72</v>
       </c>
@@ -1728,14 +1917,26 @@
       <c r="E24" t="s">
         <v>130</v>
       </c>
+      <c r="F24" t="s">
+        <v>208</v>
+      </c>
+      <c r="G24" t="s">
+        <v>213</v>
+      </c>
+      <c r="H24">
+        <v>84</v>
+      </c>
       <c r="I24" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>203</v>
       </c>
       <c r="K24" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A25" t="s">
         <v>73</v>
       </c>
@@ -1751,14 +1952,26 @@
       <c r="E25" t="s">
         <v>131</v>
       </c>
+      <c r="F25" t="s">
+        <v>208</v>
+      </c>
+      <c r="G25" t="s">
+        <v>213</v>
+      </c>
+      <c r="H25">
+        <v>84</v>
+      </c>
       <c r="I25" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>204</v>
       </c>
       <c r="K25" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46009</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -1781,7 +1994,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -1804,7 +2017,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A28" t="s">
         <v>76</v>
       </c>
@@ -1827,7 +2040,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A29" t="s">
         <v>77</v>
       </c>
@@ -1850,7 +2063,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A30" t="s">
         <v>78</v>
       </c>
@@ -1873,7 +2086,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A31" t="s">
         <v>79</v>
       </c>
@@ -1896,7 +2109,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A32" t="s">
         <v>80</v>
       </c>
@@ -1919,7 +2132,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A33" t="s">
         <v>81</v>
       </c>
@@ -1942,7 +2155,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A34" t="s">
         <v>82</v>
       </c>
@@ -1965,7 +2178,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A35" t="s">
         <v>83</v>
       </c>
@@ -1988,7 +2201,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A36" t="s">
         <v>84</v>
       </c>
@@ -2011,7 +2224,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A37" t="s">
         <v>85</v>
       </c>
@@ -2034,7 +2247,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A38" t="s">
         <v>86</v>
       </c>
@@ -2057,7 +2270,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A39" t="s">
         <v>87</v>
       </c>
@@ -2080,7 +2293,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A40" t="s">
         <v>88</v>
       </c>
@@ -2103,7 +2316,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A41" t="s">
         <v>89</v>
       </c>
@@ -2126,7 +2339,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A42" t="s">
         <v>90</v>
       </c>
@@ -2149,7 +2362,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A43" t="s">
         <v>91</v>
       </c>
@@ -2172,7 +2385,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A44" t="s">
         <v>92</v>
       </c>
@@ -2195,7 +2408,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A45" t="s">
         <v>93</v>
       </c>
@@ -2218,7 +2431,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A46" t="s">
         <v>94</v>
       </c>
@@ -2241,7 +2454,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A47" t="s">
         <v>95</v>
       </c>
@@ -2264,7 +2477,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A48" t="s">
         <v>96</v>
       </c>
@@ -2287,7 +2500,7 @@
         <v>45973</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A49" t="s">
         <v>97</v>
       </c>
@@ -2324,6 +2537,18 @@
     <hyperlink ref="J3" r:id="rId10" xr:uid="{642AF2ED-DF1B-4C99-811E-B1950408D11F}"/>
     <hyperlink ref="J13" r:id="rId11" xr:uid="{CE31A3EA-CA0D-4D7A-AA8D-0BFCA3CB5A8A}"/>
     <hyperlink ref="J2" r:id="rId12" xr:uid="{4B055461-9FA0-4B2F-AD8C-991B813205C3}"/>
+    <hyperlink ref="J14" r:id="rId13" xr:uid="{303AF4C5-9E1B-4EAE-BCEE-A2903D26B675}"/>
+    <hyperlink ref="J15" r:id="rId14" xr:uid="{72E68EE5-C196-4AD5-AEAC-53858FF4031A}"/>
+    <hyperlink ref="J16" r:id="rId15" xr:uid="{D8FF6D05-8081-4656-9D35-DB626F6D624A}"/>
+    <hyperlink ref="J17" r:id="rId16" xr:uid="{C7853AE9-38E1-4451-BD13-07E858BDD67A}"/>
+    <hyperlink ref="J18" r:id="rId17" xr:uid="{DA6AFA57-8A43-4942-8FA0-3BAFDC2A4189}"/>
+    <hyperlink ref="J19" r:id="rId18" xr:uid="{59E9D612-1287-47B5-84B6-36CECDD5EFC4}"/>
+    <hyperlink ref="J20" r:id="rId19" xr:uid="{AF83533D-EDCF-4DD4-88B0-892157BC74F4}"/>
+    <hyperlink ref="J21" r:id="rId20" xr:uid="{3C52C5BE-2B63-4419-8854-599DE62A5899}"/>
+    <hyperlink ref="J22" r:id="rId21" xr:uid="{0CE6BA49-4CEA-43D7-9291-2C82F4F8ECC0}"/>
+    <hyperlink ref="J23" r:id="rId22" xr:uid="{FDEC6D9B-3C08-4229-B3BE-54087A9AEE78}"/>
+    <hyperlink ref="J24" r:id="rId23" xr:uid="{8334CE95-AD9B-47AC-A89F-84990CC8047F}"/>
+    <hyperlink ref="J25" r:id="rId24" xr:uid="{C6874F73-79F0-436F-BE82-814FE31469E2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
requirements_traceability.xlsx updated with Sprint 3 & 4 stories
</commit_message>
<xml_diff>
--- a/Evidence/REQM/requirements_traceability.xlsx
+++ b/Evidence/REQM/requirements_traceability.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095\Evidence\REQM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA06A936-E665-4354-8B47-D826D6D9F425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF63847-CB36-4A23-8BBC-E186AA5F8B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="16186" xr2:uid="{69E9F38F-E908-4412-9BBE-056D5BFD6B03}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="203">
   <si>
     <t>Story ID</t>
   </si>
@@ -176,9 +176,6 @@
     <t>As a user, I want to view detailed playback statistics (total listening time, most-played artists) so that I can understand my listening habits.</t>
   </si>
   <si>
-    <t>As a user, I want the player to watch my music folders for file changes so that my library stays accurate without manual scans.</t>
-  </si>
-  <si>
     <t>As a user, I want to export a playlist as a text/CSV file so that I can share it with others or open it somewhere else.</t>
   </si>
   <si>
@@ -341,15 +338,9 @@
     <t>Must</t>
   </si>
   <si>
-    <t>Acceptance Criteria Summary</t>
-  </si>
-  <si>
     <t>Code Modules / Files</t>
   </si>
   <si>
-    <t>Test Cases / Files</t>
-  </si>
-  <si>
     <t>Coverage %</t>
   </si>
   <si>
@@ -365,153 +356,6 @@
     <t>Should</t>
   </si>
   <si>
-    <t>play starts/resumes; pause toggles; stop halts &amp; resets; errors handled; state reflected in UI</t>
-  </si>
-  <si>
-    <t>next advances; prev goes back; wrap behavior; single/empty list handling</t>
-  </si>
-  <si>
-    <t>shows title/artist/duration; updates on change; fallback to filename; formatting</t>
-  </si>
-  <si>
-    <t>displays elapsed/total; updates each second; paused stops increment; unknown duration handled</t>
-  </si>
-  <si>
-    <t>text bar matches position; parse mm:ss or seconds; clamp to range; state preserved</t>
-  </si>
-  <si>
-    <t>maps keys; works when UI focused; conflicts handled; repeat-safe</t>
-  </si>
-  <si>
-    <t>ff adds 5s; rw subtracts 5s; clamps; works in paused/playing</t>
-  </si>
-  <si>
-    <t>toggle mute; remember previous volume; set volume while muted updates stored value</t>
-  </si>
-  <si>
-    <t>current track prefixed icon; updates on state changes; accurate index mapping</t>
-  </si>
-  <si>
-    <t>help lists commands &amp; descriptions; help &lt;cmd&gt; shows detail; unknown suggests help</t>
-  </si>
-  <si>
-    <t>separate playback thread/task; CLI non-blocking; graceful shutdown; resource cleanup</t>
-  </si>
-  <si>
-    <t>create playlist; rename existing; delete by name/id; errors for duplicates/not found</t>
-  </si>
-  <si>
-    <t>add by id/path; remove by index/id; reorder by move/swap; persistence</t>
-  </si>
-  <si>
-    <t>case-insensitive search; partial matches; multiple fields; empty result handled</t>
-  </si>
-  <si>
-    <t>tabular layout; columns aligned; pagination if needed; null-safe values</t>
-  </si>
-  <si>
-    <t>list with name &amp; count; select by name/number; errors for invalid</t>
-  </si>
-  <si>
-    <t>show numbered tracks with durations; handles empty; updates on changes</t>
-  </si>
-  <si>
-    <t>add by search result/id; confirm existence; prevent duplicates (or allow as option)</t>
-  </si>
-  <si>
-    <t>success messages include playlist &amp; song; failures include reason; no silent errors</t>
-  </si>
-  <si>
-    <t>scan path recursively; supported extensions only; update library; handle duplicates</t>
-  </si>
-  <si>
-    <t>shows track count and hh:mm:ss; recalculates on change; accurate sum</t>
-  </si>
-  <si>
-    <t>merge A+B; optional remove duplicates; stable order; returns new playlist</t>
-  </si>
-  <si>
-    <t>deep copy retains order; new name required; independent edits</t>
-  </si>
-  <si>
-    <t>toggle shuffle; deterministic with seed; persists state; respects queue</t>
-  </si>
-  <si>
-    <t>loop single track; loop playlist; off state; interactions with next/prev</t>
-  </si>
-  <si>
-    <t>show current queue order; show history list; empty states handled</t>
-  </si>
-  <si>
-    <t>enqueue by id; remove by position/id; no duplicates optional; immediate effect</t>
-  </si>
-  <si>
-    <t>place song at position 1 in queue; respects currently playing; id validation</t>
-  </si>
-  <si>
-    <t>one command clears queue; playback unaffected until next track; confirm message</t>
-  </si>
-  <si>
-    <t>list all liked tracks; sort by date liked or title; empty state handled</t>
-  </si>
-  <si>
-    <t>sort by chosen key; stable sort; reversible; persists order</t>
-  </si>
-  <si>
-    <t>track play counts; list top N; ties deterministic</t>
-  </si>
-  <si>
-    <t>set timer minutes; cancels/overrides; stops playback on expiry; persistence optional</t>
-  </si>
-  <si>
-    <t>persist on exit; load on start; defaults if file missing; error-tolerant</t>
-  </si>
-  <si>
-    <t>define schedules; next-run calculation; execute play at time; overlap handling</t>
-  </si>
-  <si>
-    <t>checkpoint periodically; restore on start; file corruption safe</t>
-  </si>
-  <si>
-    <t>create tags; assign to songs; filter query (AND/OR/basic); persist</t>
-  </si>
-  <si>
-    <t>list by added timestamp; configurable window; empty state handled</t>
-  </si>
-  <si>
-    <t>create/switch profiles; isolated settings/library/playlists; default profile</t>
-  </si>
-  <si>
-    <t>accumulate per track/artist; total listening time; render stats view</t>
-  </si>
-  <si>
-    <t>export fields index/title/artist/duration/path; write CSV; handle IO errors</t>
-  </si>
-  <si>
-    <t>accepts numeric input; clamps 0-100; errors for invalid; immediate effect</t>
-  </si>
-  <si>
-    <t>set rating 1-10; filter by rating; auto playlists per rating</t>
-  </si>
-  <si>
-    <t>edit fields; validation; data persists</t>
-  </si>
-  <si>
-    <t>add/remove changed files; robustness to rapid changes</t>
-  </si>
-  <si>
-    <t>import local/external; skip unsupported; duplicate; progress reporting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">toggle like; persist per track; </t>
-  </si>
-  <si>
-    <t>accept 0.5-2.0; clamp; persists; affects playback timing</t>
-  </si>
-  <si>
-    <t>Backlog</t>
-  </si>
-  <si>
     <t>player_core.py, player_state.py</t>
   </si>
   <si>
@@ -678,6 +522,129 @@
   </si>
   <si>
     <t>test_music_player_playlists_advanced.py, test_np343_blackbox_specification_playlists_advanced.py, test_whitebox_playlists_advanced_branch.py, test_whitebox_playlists_advanced_statement.py</t>
+  </si>
+  <si>
+    <t>player_core.py, player_queue.py</t>
+  </si>
+  <si>
+    <t>player_metrics.py</t>
+  </si>
+  <si>
+    <t>player_config.py</t>
+  </si>
+  <si>
+    <t>player_time.py</t>
+  </si>
+  <si>
+    <t>player_io.py</t>
+  </si>
+  <si>
+    <t>user_data.py</t>
+  </si>
+  <si>
+    <t>As a user, I want to perform advanced searches (e.g. artist:NAME, duration&lt;3:00) so that I can filter my library more specifically.</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-01-shuffle-mode-on-off</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-02-loop-mode</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-28-current-queue-recently-played</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-04-add-or-remove-songs-from-queue</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-05-queue-specific-song-to-play-next</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-06-clear-queue</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-07-playback-speed</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-08-like-or-unlike-song</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-09-view-liked-songs</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-10-sort-playlists</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-11-most-played-songs</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S3-12-sleep-timer</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-01-save-settings</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-02-schedule-playback</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-03-last-song-position</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-04-import-songs</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-05-custom-tags</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-06-recently-added</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-07-user-profile-switch</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-08-playback-stats</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-09-advanced-search</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-10-export-playlist</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-11-update-metadata</t>
+  </si>
+  <si>
+    <t>https://github.com/neelpatkar007/CO3095-Group-16-Music-Player-Application/tree/feature/S4-12-rate-songs</t>
+  </si>
+  <si>
+    <t>test_music_player_player_queue.py, test_player_queue_branch.py</t>
+  </si>
+  <si>
+    <t>Test Files</t>
+  </si>
+  <si>
+    <t>test_music_player_player_queue.py, test_player_queue_branch.py, test_music_player_player_core.py, test_player_core.py, test_player_core_branch.py, test_player_core_statement.py</t>
+  </si>
+  <si>
+    <t>test_music_player_player_core.py, test_player_core.py, test_player_core_branch.py, test_player_core_statement.py</t>
+  </si>
+  <si>
+    <t>test_music_player_playlists_basic.py, test_playlists_basic.py, test_playlists_basic_branch.py, test_playlists_basic_statement.py</t>
+  </si>
+  <si>
+    <t>test_music_player_player_metrics.py, test_player_metrics.py</t>
+  </si>
+  <si>
+    <t>test_player_io.py</t>
+  </si>
+  <si>
+    <t>test_music_player_player_config.py, test_player_config.py, test_player_config_branch.py, test_player_config_statement.py</t>
+  </si>
+  <si>
+    <t>test_music_player_user_data.py, test_user_data_branch.py, test_user_data_statement.py</t>
+  </si>
+  <si>
+    <t>test_music_player_player_time.py, test_player_time.py, test_player_time_branch.py</t>
   </si>
 </sst>
 </file>
@@ -1079,23 +1046,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C023A292-D7D7-42AA-A66D-EAC889642A87}">
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="2" max="2" width="146.87890625" customWidth="1"/>
     <col min="3" max="3" width="6.87890625" customWidth="1"/>
     <col min="4" max="4" width="19.29296875" customWidth="1"/>
-    <col min="5" max="5" width="88.41015625" customWidth="1"/>
-    <col min="6" max="6" width="29.41015625" customWidth="1"/>
-    <col min="7" max="7" width="236.29296875" customWidth="1"/>
-    <col min="8" max="8" width="12.5859375" customWidth="1"/>
-    <col min="9" max="9" width="12.703125" customWidth="1"/>
-    <col min="10" max="10" width="118.5859375" customWidth="1"/>
-    <col min="11" max="11" width="13.1171875" customWidth="1"/>
-    <col min="12" max="12" width="14.1171875" customWidth="1"/>
+    <col min="5" max="5" width="29.41015625" customWidth="1"/>
+    <col min="6" max="6" width="236.29296875" customWidth="1"/>
+    <col min="7" max="7" width="12.5859375" customWidth="1"/>
+    <col min="8" max="8" width="12.703125" customWidth="1"/>
+    <col min="9" max="9" width="118.5859375" customWidth="1"/>
+    <col min="10" max="10" width="13.1171875" customWidth="1"/>
+    <col min="11" max="11" width="14.1171875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1103,37 +1069,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>99</v>
-      </c>
       <c r="E1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1" s="1"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -1142,33 +1105,30 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G2">
         <v>100</v>
       </c>
-      <c r="E2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F2" t="s">
-        <v>158</v>
-      </c>
-      <c r="G2" t="s">
-        <v>179</v>
-      </c>
-      <c r="H2">
-        <v>100</v>
-      </c>
-      <c r="I2" t="s">
-        <v>192</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="K2" s="3">
+      <c r="H2" t="s">
+        <v>140</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="J2" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>3</v>
@@ -1177,33 +1137,30 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="F3" t="s">
-        <v>159</v>
-      </c>
-      <c r="G3" t="s">
-        <v>180</v>
-      </c>
-      <c r="H3">
+        <v>128</v>
+      </c>
+      <c r="G3">
         <v>75</v>
       </c>
-      <c r="I3" t="s">
-        <v>192</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="K3" s="3">
+      <c r="H3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="J3" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>
@@ -1212,33 +1169,30 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4">
         <v>100</v>
       </c>
-      <c r="E4" t="s">
-        <v>111</v>
-      </c>
-      <c r="F4" t="s">
-        <v>160</v>
-      </c>
-      <c r="G4" t="s">
-        <v>181</v>
-      </c>
-      <c r="H4">
-        <v>100</v>
-      </c>
-      <c r="I4" t="s">
-        <v>192</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="K4" s="3">
+      <c r="H4" t="s">
+        <v>140</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J4" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>5</v>
@@ -1247,33 +1201,30 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F5" t="s">
+        <v>130</v>
+      </c>
+      <c r="G5">
         <v>100</v>
       </c>
-      <c r="E5" t="s">
-        <v>150</v>
-      </c>
-      <c r="F5" t="s">
-        <v>161</v>
-      </c>
-      <c r="G5" t="s">
-        <v>182</v>
-      </c>
-      <c r="H5">
-        <v>100</v>
-      </c>
-      <c r="I5" t="s">
-        <v>192</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="K5" s="3">
+      <c r="H5" t="s">
+        <v>140</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="J5" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>6</v>
@@ -1282,33 +1233,30 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F6" t="s">
+        <v>131</v>
+      </c>
+      <c r="G6">
         <v>100</v>
       </c>
-      <c r="E6" t="s">
-        <v>112</v>
-      </c>
-      <c r="F6" t="s">
-        <v>163</v>
-      </c>
-      <c r="G6" t="s">
-        <v>183</v>
-      </c>
-      <c r="H6">
-        <v>100</v>
-      </c>
-      <c r="I6" t="s">
-        <v>192</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="K6" s="3">
+      <c r="H6" t="s">
+        <v>140</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="J6" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
@@ -1317,33 +1265,30 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G7">
         <v>100</v>
       </c>
-      <c r="E7" t="s">
-        <v>113</v>
-      </c>
-      <c r="F7" t="s">
-        <v>162</v>
-      </c>
-      <c r="G7" t="s">
-        <v>184</v>
-      </c>
-      <c r="H7">
-        <v>100</v>
-      </c>
-      <c r="I7" t="s">
-        <v>192</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="K7" s="3">
+      <c r="H7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="J7" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
@@ -1352,33 +1297,30 @@
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F8" t="s">
-        <v>164</v>
-      </c>
-      <c r="G8" t="s">
-        <v>185</v>
-      </c>
-      <c r="H8">
+        <v>133</v>
+      </c>
+      <c r="G8">
         <v>100</v>
       </c>
-      <c r="I8" t="s">
-        <v>192</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="K8" s="3">
+      <c r="H8" t="s">
+        <v>140</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="J8" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>9</v>
@@ -1387,33 +1329,30 @@
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E9" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F9" t="s">
-        <v>162</v>
-      </c>
-      <c r="G9" t="s">
-        <v>186</v>
-      </c>
-      <c r="H9">
+        <v>134</v>
+      </c>
+      <c r="G9">
         <v>100</v>
       </c>
-      <c r="I9" t="s">
-        <v>192</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="K9" s="3">
+      <c r="H9" t="s">
+        <v>140</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="J9" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>10</v>
@@ -1422,33 +1361,30 @@
         <v>1</v>
       </c>
       <c r="D10" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" t="s">
+        <v>109</v>
+      </c>
+      <c r="F10" t="s">
+        <v>135</v>
+      </c>
+      <c r="G10">
         <v>100</v>
       </c>
-      <c r="E10" t="s">
-        <v>116</v>
-      </c>
-      <c r="F10" t="s">
-        <v>161</v>
-      </c>
-      <c r="G10" t="s">
-        <v>187</v>
-      </c>
-      <c r="H10">
-        <v>100</v>
-      </c>
-      <c r="I10" t="s">
-        <v>192</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="K10" s="3">
+      <c r="H10" t="s">
+        <v>140</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="J10" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>11</v>
@@ -1457,33 +1393,30 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E11" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="F11" t="s">
-        <v>163</v>
-      </c>
-      <c r="G11" t="s">
-        <v>188</v>
-      </c>
-      <c r="H11">
+        <v>136</v>
+      </c>
+      <c r="G11">
         <v>93</v>
       </c>
-      <c r="I11" t="s">
-        <v>192</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="K11" s="3">
+      <c r="H11" t="s">
+        <v>140</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="J11" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
@@ -1492,33 +1425,30 @@
         <v>1</v>
       </c>
       <c r="D12" t="s">
+        <v>99</v>
+      </c>
+      <c r="E12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F12" t="s">
+        <v>137</v>
+      </c>
+      <c r="G12">
         <v>100</v>
       </c>
-      <c r="E12" t="s">
-        <v>118</v>
-      </c>
-      <c r="F12" t="s">
-        <v>165</v>
-      </c>
-      <c r="G12" t="s">
-        <v>189</v>
-      </c>
-      <c r="H12">
-        <v>100</v>
-      </c>
-      <c r="I12" t="s">
-        <v>192</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="K12" s="3">
+      <c r="H12" t="s">
+        <v>140</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="J12" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>13</v>
@@ -1527,33 +1457,30 @@
         <v>1</v>
       </c>
       <c r="D13" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" t="s">
+        <v>114</v>
+      </c>
+      <c r="F13" t="s">
+        <v>138</v>
+      </c>
+      <c r="G13">
         <v>100</v>
       </c>
-      <c r="E13" t="s">
-        <v>119</v>
-      </c>
-      <c r="F13" t="s">
-        <v>166</v>
-      </c>
-      <c r="G13" t="s">
-        <v>190</v>
-      </c>
-      <c r="H13">
-        <v>100</v>
-      </c>
-      <c r="I13" t="s">
-        <v>192</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="K13" s="3">
+      <c r="H13" t="s">
+        <v>140</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="J13" s="3">
         <v>45993</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>25</v>
@@ -1562,33 +1489,30 @@
         <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E14" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="F14" t="s">
-        <v>191</v>
-      </c>
-      <c r="G14" t="s">
-        <v>209</v>
-      </c>
-      <c r="H14">
+        <v>157</v>
+      </c>
+      <c r="G14">
         <v>89</v>
       </c>
-      <c r="I14" t="s">
-        <v>192</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="K14" s="3">
+      <c r="H14" t="s">
+        <v>140</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="J14" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>24</v>
@@ -1597,33 +1521,30 @@
         <v>2</v>
       </c>
       <c r="D15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E15" t="s">
-        <v>121</v>
+        <v>153</v>
       </c>
       <c r="F15" t="s">
-        <v>205</v>
-      </c>
-      <c r="G15" t="s">
-        <v>211</v>
-      </c>
-      <c r="H15">
+        <v>159</v>
+      </c>
+      <c r="G15">
         <v>99</v>
       </c>
-      <c r="I15" t="s">
-        <v>192</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="K15" s="3">
+      <c r="H15" t="s">
+        <v>140</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="J15" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>23</v>
@@ -1632,33 +1553,30 @@
         <v>2</v>
       </c>
       <c r="D16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E16" t="s">
-        <v>122</v>
+        <v>154</v>
       </c>
       <c r="F16" t="s">
-        <v>206</v>
-      </c>
-      <c r="G16" t="s">
-        <v>212</v>
-      </c>
-      <c r="H16">
+        <v>160</v>
+      </c>
+      <c r="G16">
         <v>97</v>
       </c>
-      <c r="I16" t="s">
-        <v>192</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="K16" s="3">
+      <c r="H16" t="s">
+        <v>140</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="J16" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>22</v>
@@ -1667,33 +1585,30 @@
         <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E17" t="s">
-        <v>123</v>
+        <v>154</v>
       </c>
       <c r="F17" t="s">
-        <v>206</v>
-      </c>
-      <c r="G17" t="s">
-        <v>212</v>
-      </c>
-      <c r="H17">
+        <v>160</v>
+      </c>
+      <c r="G17">
         <v>97</v>
       </c>
-      <c r="I17" t="s">
-        <v>192</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="K17" s="3">
+      <c r="H17" t="s">
+        <v>140</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="J17" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>21</v>
@@ -1702,33 +1617,30 @@
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E18" t="s">
-        <v>124</v>
+        <v>155</v>
       </c>
       <c r="F18" t="s">
-        <v>207</v>
-      </c>
-      <c r="G18" t="s">
-        <v>210</v>
-      </c>
-      <c r="H18">
+        <v>158</v>
+      </c>
+      <c r="G18">
         <v>89</v>
       </c>
-      <c r="I18" t="s">
-        <v>192</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="K18" s="3">
+      <c r="H18" t="s">
+        <v>140</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="J18" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>20</v>
@@ -1737,33 +1649,30 @@
         <v>2</v>
       </c>
       <c r="D19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E19" t="s">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="F19" t="s">
-        <v>207</v>
-      </c>
-      <c r="G19" t="s">
-        <v>210</v>
-      </c>
-      <c r="H19">
+        <v>158</v>
+      </c>
+      <c r="G19">
         <v>89</v>
       </c>
-      <c r="I19" t="s">
-        <v>192</v>
-      </c>
-      <c r="J19" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="K19" s="3">
+      <c r="H19" t="s">
+        <v>140</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="J19" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>19</v>
@@ -1772,33 +1681,30 @@
         <v>2</v>
       </c>
       <c r="D20" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E20" t="s">
-        <v>126</v>
+        <v>153</v>
       </c>
       <c r="F20" t="s">
-        <v>205</v>
-      </c>
-      <c r="G20" t="s">
-        <v>211</v>
-      </c>
-      <c r="H20">
+        <v>159</v>
+      </c>
+      <c r="G20">
         <v>99</v>
       </c>
-      <c r="I20" t="s">
-        <v>192</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="K20" s="3">
+      <c r="H20" t="s">
+        <v>140</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="J20" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>18</v>
@@ -1807,33 +1713,30 @@
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E21" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="F21" t="s">
-        <v>205</v>
-      </c>
-      <c r="G21" t="s">
-        <v>211</v>
-      </c>
-      <c r="H21">
+        <v>159</v>
+      </c>
+      <c r="G21">
         <v>99</v>
       </c>
-      <c r="I21" t="s">
-        <v>192</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="K21" s="3">
+      <c r="H21" t="s">
+        <v>140</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="J21" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A22" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>17</v>
@@ -1842,33 +1745,30 @@
         <v>2</v>
       </c>
       <c r="D22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E22" t="s">
-        <v>128</v>
+        <v>154</v>
       </c>
       <c r="F22" t="s">
-        <v>206</v>
-      </c>
-      <c r="G22" t="s">
-        <v>212</v>
-      </c>
-      <c r="H22">
+        <v>160</v>
+      </c>
+      <c r="G22">
         <v>97</v>
       </c>
-      <c r="I22" t="s">
-        <v>192</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="K22" s="3">
+      <c r="H22" t="s">
+        <v>140</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="J22" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>16</v>
@@ -1877,33 +1777,30 @@
         <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E23" t="s">
-        <v>129</v>
+        <v>155</v>
       </c>
       <c r="F23" t="s">
-        <v>207</v>
-      </c>
-      <c r="G23" t="s">
-        <v>210</v>
-      </c>
-      <c r="H23">
+        <v>158</v>
+      </c>
+      <c r="G23">
         <v>89</v>
       </c>
-      <c r="I23" t="s">
-        <v>192</v>
-      </c>
-      <c r="J23" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="K23" s="3">
+      <c r="H23" t="s">
+        <v>140</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="J23" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A24" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>15</v>
@@ -1912,33 +1809,30 @@
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E24" t="s">
-        <v>130</v>
+        <v>156</v>
       </c>
       <c r="F24" t="s">
-        <v>208</v>
-      </c>
-      <c r="G24" t="s">
-        <v>213</v>
-      </c>
-      <c r="H24">
+        <v>161</v>
+      </c>
+      <c r="G24">
         <v>84</v>
       </c>
-      <c r="I24" t="s">
-        <v>192</v>
-      </c>
-      <c r="J24" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="K24" s="3">
+      <c r="H24" t="s">
+        <v>140</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J24" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>14</v>
@@ -1947,33 +1841,30 @@
         <v>2</v>
       </c>
       <c r="D25" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E25" t="s">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="F25" t="s">
-        <v>208</v>
-      </c>
-      <c r="G25" t="s">
-        <v>213</v>
-      </c>
-      <c r="H25">
+        <v>161</v>
+      </c>
+      <c r="G25">
         <v>84</v>
       </c>
-      <c r="I25" t="s">
-        <v>192</v>
-      </c>
-      <c r="J25" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="K25" s="3">
+      <c r="H25" t="s">
+        <v>140</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="J25" s="3">
         <v>46009</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>26</v>
@@ -1982,21 +1873,30 @@
         <v>3</v>
       </c>
       <c r="D26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E26" t="s">
-        <v>132</v>
-      </c>
-      <c r="I26" t="s">
-        <v>157</v>
-      </c>
-      <c r="K26" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.5">
+        <v>107</v>
+      </c>
+      <c r="F26" t="s">
+        <v>193</v>
+      </c>
+      <c r="G26">
+        <v>70</v>
+      </c>
+      <c r="H26" t="s">
+        <v>140</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="J26" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>27</v>
@@ -2005,21 +1905,30 @@
         <v>3</v>
       </c>
       <c r="D27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E27" t="s">
-        <v>133</v>
-      </c>
-      <c r="I27" t="s">
-        <v>157</v>
-      </c>
-      <c r="K27" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.5">
+        <v>107</v>
+      </c>
+      <c r="F27" t="s">
+        <v>193</v>
+      </c>
+      <c r="G27">
+        <v>70</v>
+      </c>
+      <c r="H27" t="s">
+        <v>140</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="J27" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>28</v>
@@ -2028,21 +1937,30 @@
         <v>3</v>
       </c>
       <c r="D28" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E28" t="s">
-        <v>134</v>
-      </c>
-      <c r="I28" t="s">
-        <v>157</v>
-      </c>
-      <c r="K28" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.5">
+        <v>107</v>
+      </c>
+      <c r="F28" t="s">
+        <v>193</v>
+      </c>
+      <c r="G28">
+        <v>70</v>
+      </c>
+      <c r="H28" t="s">
+        <v>140</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="J28" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>29</v>
@@ -2051,21 +1969,30 @@
         <v>3</v>
       </c>
       <c r="D29" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E29" t="s">
-        <v>135</v>
-      </c>
-      <c r="I29" t="s">
-        <v>157</v>
-      </c>
-      <c r="K29" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.5">
+        <v>107</v>
+      </c>
+      <c r="F29" t="s">
+        <v>193</v>
+      </c>
+      <c r="G29">
+        <v>70</v>
+      </c>
+      <c r="H29" t="s">
+        <v>140</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="J29" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>30</v>
@@ -2074,21 +2001,30 @@
         <v>3</v>
       </c>
       <c r="D30" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E30" t="s">
-        <v>136</v>
-      </c>
-      <c r="I30" t="s">
-        <v>157</v>
-      </c>
-      <c r="K30" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.5">
+        <v>107</v>
+      </c>
+      <c r="F30" t="s">
+        <v>193</v>
+      </c>
+      <c r="G30">
+        <v>70</v>
+      </c>
+      <c r="H30" t="s">
+        <v>140</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="J30" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>31</v>
@@ -2097,21 +2033,30 @@
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E31" t="s">
-        <v>137</v>
-      </c>
-      <c r="I31" t="s">
-        <v>157</v>
-      </c>
-      <c r="K31" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.5">
+        <v>107</v>
+      </c>
+      <c r="F31" t="s">
+        <v>193</v>
+      </c>
+      <c r="G31">
+        <v>70</v>
+      </c>
+      <c r="H31" t="s">
+        <v>140</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="J31" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A32" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>32</v>
@@ -2120,21 +2065,30 @@
         <v>3</v>
       </c>
       <c r="D32" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E32" t="s">
-        <v>156</v>
-      </c>
-      <c r="I32" t="s">
-        <v>157</v>
-      </c>
-      <c r="K32" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.5">
+        <v>162</v>
+      </c>
+      <c r="F32" t="s">
+        <v>195</v>
+      </c>
+      <c r="G32">
+        <v>78</v>
+      </c>
+      <c r="H32" t="s">
+        <v>140</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J32" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A33" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>33</v>
@@ -2143,21 +2097,30 @@
         <v>3</v>
       </c>
       <c r="D33" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E33" t="s">
-        <v>155</v>
-      </c>
-      <c r="I33" t="s">
-        <v>157</v>
-      </c>
-      <c r="K33" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.5">
+        <v>163</v>
+      </c>
+      <c r="F33" t="s">
+        <v>198</v>
+      </c>
+      <c r="G33">
+        <v>89</v>
+      </c>
+      <c r="H33" t="s">
+        <v>140</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="J33" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A34" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>34</v>
@@ -2166,21 +2129,30 @@
         <v>3</v>
       </c>
       <c r="D34" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E34" t="s">
-        <v>138</v>
-      </c>
-      <c r="I34" t="s">
-        <v>157</v>
-      </c>
-      <c r="K34" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.5">
+        <v>163</v>
+      </c>
+      <c r="F34" t="s">
+        <v>198</v>
+      </c>
+      <c r="G34">
+        <v>89</v>
+      </c>
+      <c r="H34" t="s">
+        <v>140</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J34" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A35" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>35</v>
@@ -2189,21 +2161,30 @@
         <v>3</v>
       </c>
       <c r="D35" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E35" t="s">
-        <v>139</v>
-      </c>
-      <c r="I35" t="s">
-        <v>157</v>
-      </c>
-      <c r="K35" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.5">
+        <v>155</v>
+      </c>
+      <c r="F35" t="s">
+        <v>197</v>
+      </c>
+      <c r="G35">
+        <v>93</v>
+      </c>
+      <c r="H35" t="s">
+        <v>140</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="J35" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>36</v>
@@ -2212,21 +2193,30 @@
         <v>3</v>
       </c>
       <c r="D36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E36" t="s">
-        <v>140</v>
-      </c>
-      <c r="I36" t="s">
-        <v>157</v>
-      </c>
-      <c r="K36" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.5">
+        <v>163</v>
+      </c>
+      <c r="F36" t="s">
+        <v>198</v>
+      </c>
+      <c r="G36">
+        <v>89</v>
+      </c>
+      <c r="H36" t="s">
+        <v>140</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="J36" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>37</v>
@@ -2235,21 +2225,30 @@
         <v>3</v>
       </c>
       <c r="D37" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E37" t="s">
-        <v>141</v>
-      </c>
-      <c r="I37" t="s">
-        <v>157</v>
-      </c>
-      <c r="K37" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.5">
+        <v>114</v>
+      </c>
+      <c r="F37" t="s">
+        <v>196</v>
+      </c>
+      <c r="G37">
+        <v>86</v>
+      </c>
+      <c r="H37" t="s">
+        <v>140</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="J37" s="3">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A38" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>38</v>
@@ -2258,21 +2257,30 @@
         <v>4</v>
       </c>
       <c r="D38" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E38" t="s">
-        <v>142</v>
-      </c>
-      <c r="I38" t="s">
-        <v>157</v>
-      </c>
-      <c r="K38" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.5">
+        <v>164</v>
+      </c>
+      <c r="F38" t="s">
+        <v>200</v>
+      </c>
+      <c r="G38">
+        <v>85</v>
+      </c>
+      <c r="H38" t="s">
+        <v>140</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="J38" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A39" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>39</v>
@@ -2281,21 +2289,30 @@
         <v>4</v>
       </c>
       <c r="D39" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E39" t="s">
-        <v>143</v>
-      </c>
-      <c r="I39" t="s">
-        <v>157</v>
-      </c>
-      <c r="K39" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.5">
+        <v>165</v>
+      </c>
+      <c r="F39" t="s">
+        <v>202</v>
+      </c>
+      <c r="G39">
+        <v>77</v>
+      </c>
+      <c r="H39" t="s">
+        <v>140</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="J39" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>40</v>
@@ -2304,21 +2321,30 @@
         <v>4</v>
       </c>
       <c r="D40" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E40" t="s">
-        <v>144</v>
-      </c>
-      <c r="I40" t="s">
-        <v>157</v>
-      </c>
-      <c r="K40" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.5">
+        <v>165</v>
+      </c>
+      <c r="F40" t="s">
+        <v>202</v>
+      </c>
+      <c r="G40">
+        <v>77</v>
+      </c>
+      <c r="H40" t="s">
+        <v>140</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="J40" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A41" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>41</v>
@@ -2327,21 +2353,30 @@
         <v>4</v>
       </c>
       <c r="D41" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E41" t="s">
-        <v>154</v>
-      </c>
-      <c r="I41" t="s">
-        <v>157</v>
-      </c>
-      <c r="K41" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.5">
+        <v>166</v>
+      </c>
+      <c r="F41" t="s">
+        <v>199</v>
+      </c>
+      <c r="G41">
+        <v>45</v>
+      </c>
+      <c r="H41" t="s">
+        <v>140</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="J41" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A42" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>42</v>
@@ -2350,21 +2385,30 @@
         <v>4</v>
       </c>
       <c r="D42" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E42" t="s">
-        <v>145</v>
-      </c>
-      <c r="I42" t="s">
-        <v>157</v>
-      </c>
-      <c r="K42" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.5">
+        <v>164</v>
+      </c>
+      <c r="F42" t="s">
+        <v>200</v>
+      </c>
+      <c r="G42">
+        <v>85</v>
+      </c>
+      <c r="H42" t="s">
+        <v>140</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="J42" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>43</v>
@@ -2373,21 +2417,30 @@
         <v>4</v>
       </c>
       <c r="D43" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E43" t="s">
-        <v>146</v>
-      </c>
-      <c r="I43" t="s">
-        <v>157</v>
-      </c>
-      <c r="K43" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.5">
+        <v>165</v>
+      </c>
+      <c r="F43" t="s">
+        <v>202</v>
+      </c>
+      <c r="G43">
+        <v>77</v>
+      </c>
+      <c r="H43" t="s">
+        <v>140</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="J43" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A44" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>44</v>
@@ -2396,21 +2449,30 @@
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E44" t="s">
-        <v>147</v>
-      </c>
-      <c r="I44" t="s">
-        <v>157</v>
-      </c>
-      <c r="K44" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.5">
+        <v>167</v>
+      </c>
+      <c r="F44" t="s">
+        <v>201</v>
+      </c>
+      <c r="G44">
+        <v>73</v>
+      </c>
+      <c r="H44" t="s">
+        <v>140</v>
+      </c>
+      <c r="I44" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="J44" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A45" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>45</v>
@@ -2419,136 +2481,205 @@
         <v>4</v>
       </c>
       <c r="D45" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E45" t="s">
-        <v>148</v>
-      </c>
-      <c r="I45" t="s">
-        <v>157</v>
-      </c>
-      <c r="K45" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.5">
+        <v>164</v>
+      </c>
+      <c r="F45" t="s">
+        <v>200</v>
+      </c>
+      <c r="G45">
+        <v>85</v>
+      </c>
+      <c r="H45" t="s">
+        <v>140</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="J45" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>46</v>
+        <v>168</v>
       </c>
       <c r="C46">
         <v>4</v>
       </c>
       <c r="D46" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E46" t="s">
-        <v>153</v>
-      </c>
-      <c r="I46" t="s">
-        <v>157</v>
-      </c>
-      <c r="K46" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.5">
+        <v>167</v>
+      </c>
+      <c r="F46" t="s">
+        <v>201</v>
+      </c>
+      <c r="G46">
+        <v>73</v>
+      </c>
+      <c r="H46" t="s">
+        <v>140</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="J46" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A47" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C47">
         <v>4</v>
       </c>
       <c r="D47" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E47" t="s">
-        <v>149</v>
-      </c>
-      <c r="I47" t="s">
-        <v>157</v>
-      </c>
-      <c r="K47" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.5">
+        <v>166</v>
+      </c>
+      <c r="F47" t="s">
+        <v>199</v>
+      </c>
+      <c r="G47">
+        <v>45</v>
+      </c>
+      <c r="H47" t="s">
+        <v>140</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="J47" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A48" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C48">
         <v>4</v>
       </c>
       <c r="D48" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E48" t="s">
-        <v>152</v>
-      </c>
-      <c r="I48" t="s">
-        <v>157</v>
-      </c>
-      <c r="K48" s="3">
-        <v>45973</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.5">
+        <v>166</v>
+      </c>
+      <c r="F48" t="s">
+        <v>199</v>
+      </c>
+      <c r="G48">
+        <v>45</v>
+      </c>
+      <c r="H48" t="s">
+        <v>140</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J48" s="3">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A49" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C49">
         <v>4</v>
       </c>
       <c r="D49" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E49" t="s">
-        <v>151</v>
-      </c>
-      <c r="I49" t="s">
-        <v>157</v>
-      </c>
-      <c r="K49" s="3">
-        <v>45973</v>
+        <v>167</v>
+      </c>
+      <c r="F49" t="s">
+        <v>201</v>
+      </c>
+      <c r="G49">
+        <v>73</v>
+      </c>
+      <c r="H49" t="s">
+        <v>140</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="J49" s="3">
+        <v>46025</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J12" r:id="rId1" xr:uid="{3F8D44C8-F061-4367-B70C-9D38E43EEBF7}"/>
-    <hyperlink ref="J7" r:id="rId2" xr:uid="{07BB3D38-21FE-48F7-BA31-D9360AC2C1B2}"/>
-    <hyperlink ref="J10" r:id="rId3" xr:uid="{98B5085D-BC3C-4BA5-8B6A-C6640DAAE840}"/>
-    <hyperlink ref="J6" r:id="rId4" xr:uid="{345855EB-85A7-432D-B808-7548D6CED3EC}"/>
-    <hyperlink ref="J5" r:id="rId5" xr:uid="{CE4744A3-7888-4906-B759-E25B3A066C41}"/>
-    <hyperlink ref="J9" r:id="rId6" xr:uid="{A4A738A8-5311-405A-AB9A-699DDFE42174}"/>
-    <hyperlink ref="J8" r:id="rId7" xr:uid="{426ED8E3-B37E-40E8-9A3B-ABA8F1ABD897}"/>
-    <hyperlink ref="J11" r:id="rId8" xr:uid="{E6BF8555-C0F9-42F4-9D5F-9027F3F5FB4D}"/>
-    <hyperlink ref="J4" r:id="rId9" xr:uid="{75425B77-CF9D-4BC4-B354-1DED57CE5F7B}"/>
-    <hyperlink ref="J3" r:id="rId10" xr:uid="{642AF2ED-DF1B-4C99-811E-B1950408D11F}"/>
-    <hyperlink ref="J13" r:id="rId11" xr:uid="{CE31A3EA-CA0D-4D7A-AA8D-0BFCA3CB5A8A}"/>
-    <hyperlink ref="J2" r:id="rId12" xr:uid="{4B055461-9FA0-4B2F-AD8C-991B813205C3}"/>
-    <hyperlink ref="J14" r:id="rId13" xr:uid="{303AF4C5-9E1B-4EAE-BCEE-A2903D26B675}"/>
-    <hyperlink ref="J15" r:id="rId14" xr:uid="{72E68EE5-C196-4AD5-AEAC-53858FF4031A}"/>
-    <hyperlink ref="J16" r:id="rId15" xr:uid="{D8FF6D05-8081-4656-9D35-DB626F6D624A}"/>
-    <hyperlink ref="J17" r:id="rId16" xr:uid="{C7853AE9-38E1-4451-BD13-07E858BDD67A}"/>
-    <hyperlink ref="J18" r:id="rId17" xr:uid="{DA6AFA57-8A43-4942-8FA0-3BAFDC2A4189}"/>
-    <hyperlink ref="J19" r:id="rId18" xr:uid="{59E9D612-1287-47B5-84B6-36CECDD5EFC4}"/>
-    <hyperlink ref="J20" r:id="rId19" xr:uid="{AF83533D-EDCF-4DD4-88B0-892157BC74F4}"/>
-    <hyperlink ref="J21" r:id="rId20" xr:uid="{3C52C5BE-2B63-4419-8854-599DE62A5899}"/>
-    <hyperlink ref="J22" r:id="rId21" xr:uid="{0CE6BA49-4CEA-43D7-9291-2C82F4F8ECC0}"/>
-    <hyperlink ref="J23" r:id="rId22" xr:uid="{FDEC6D9B-3C08-4229-B3BE-54087A9AEE78}"/>
-    <hyperlink ref="J24" r:id="rId23" xr:uid="{8334CE95-AD9B-47AC-A89F-84990CC8047F}"/>
-    <hyperlink ref="J25" r:id="rId24" xr:uid="{C6874F73-79F0-436F-BE82-814FE31469E2}"/>
+    <hyperlink ref="I12" r:id="rId1" xr:uid="{3F8D44C8-F061-4367-B70C-9D38E43EEBF7}"/>
+    <hyperlink ref="I7" r:id="rId2" xr:uid="{07BB3D38-21FE-48F7-BA31-D9360AC2C1B2}"/>
+    <hyperlink ref="I10" r:id="rId3" xr:uid="{98B5085D-BC3C-4BA5-8B6A-C6640DAAE840}"/>
+    <hyperlink ref="I6" r:id="rId4" xr:uid="{345855EB-85A7-432D-B808-7548D6CED3EC}"/>
+    <hyperlink ref="I5" r:id="rId5" xr:uid="{CE4744A3-7888-4906-B759-E25B3A066C41}"/>
+    <hyperlink ref="I9" r:id="rId6" xr:uid="{A4A738A8-5311-405A-AB9A-699DDFE42174}"/>
+    <hyperlink ref="I8" r:id="rId7" xr:uid="{426ED8E3-B37E-40E8-9A3B-ABA8F1ABD897}"/>
+    <hyperlink ref="I11" r:id="rId8" xr:uid="{E6BF8555-C0F9-42F4-9D5F-9027F3F5FB4D}"/>
+    <hyperlink ref="I4" r:id="rId9" xr:uid="{75425B77-CF9D-4BC4-B354-1DED57CE5F7B}"/>
+    <hyperlink ref="I3" r:id="rId10" xr:uid="{642AF2ED-DF1B-4C99-811E-B1950408D11F}"/>
+    <hyperlink ref="I13" r:id="rId11" xr:uid="{CE31A3EA-CA0D-4D7A-AA8D-0BFCA3CB5A8A}"/>
+    <hyperlink ref="I2" r:id="rId12" xr:uid="{4B055461-9FA0-4B2F-AD8C-991B813205C3}"/>
+    <hyperlink ref="I14" r:id="rId13" xr:uid="{303AF4C5-9E1B-4EAE-BCEE-A2903D26B675}"/>
+    <hyperlink ref="I15" r:id="rId14" xr:uid="{72E68EE5-C196-4AD5-AEAC-53858FF4031A}"/>
+    <hyperlink ref="I16" r:id="rId15" xr:uid="{D8FF6D05-8081-4656-9D35-DB626F6D624A}"/>
+    <hyperlink ref="I17" r:id="rId16" xr:uid="{C7853AE9-38E1-4451-BD13-07E858BDD67A}"/>
+    <hyperlink ref="I18" r:id="rId17" xr:uid="{DA6AFA57-8A43-4942-8FA0-3BAFDC2A4189}"/>
+    <hyperlink ref="I19" r:id="rId18" xr:uid="{59E9D612-1287-47B5-84B6-36CECDD5EFC4}"/>
+    <hyperlink ref="I20" r:id="rId19" xr:uid="{AF83533D-EDCF-4DD4-88B0-892157BC74F4}"/>
+    <hyperlink ref="I21" r:id="rId20" xr:uid="{3C52C5BE-2B63-4419-8854-599DE62A5899}"/>
+    <hyperlink ref="I22" r:id="rId21" xr:uid="{0CE6BA49-4CEA-43D7-9291-2C82F4F8ECC0}"/>
+    <hyperlink ref="I23" r:id="rId22" xr:uid="{FDEC6D9B-3C08-4229-B3BE-54087A9AEE78}"/>
+    <hyperlink ref="I24" r:id="rId23" xr:uid="{8334CE95-AD9B-47AC-A89F-84990CC8047F}"/>
+    <hyperlink ref="I25" r:id="rId24" xr:uid="{C6874F73-79F0-436F-BE82-814FE31469E2}"/>
+    <hyperlink ref="I26" r:id="rId25" xr:uid="{2427D59C-59C8-4F18-9AEE-A42FF23CD395}"/>
+    <hyperlink ref="I27" r:id="rId26" xr:uid="{C770F842-000F-48F0-B042-B009439CCD8E}"/>
+    <hyperlink ref="I28" r:id="rId27" xr:uid="{98674C65-D7F7-44E7-A0BF-D0FA3EC8031D}"/>
+    <hyperlink ref="I29" r:id="rId28" xr:uid="{B394C4F1-9E17-428E-B09F-0BD23FA28923}"/>
+    <hyperlink ref="I30" r:id="rId29" xr:uid="{BAE3A26D-79CC-478F-8DB1-51067C6A9832}"/>
+    <hyperlink ref="I31" r:id="rId30" xr:uid="{581AA705-EC2A-4321-A799-E3F6C0386754}"/>
+    <hyperlink ref="I32" r:id="rId31" xr:uid="{986BFD9D-B3F4-44A3-8CD0-39164893296E}"/>
+    <hyperlink ref="I33" r:id="rId32" xr:uid="{0786BD41-D119-4F44-85F2-34DA84CD5DC6}"/>
+    <hyperlink ref="I34" r:id="rId33" xr:uid="{EDC528D6-96B9-400E-B57C-DC6A6F991211}"/>
+    <hyperlink ref="I35" r:id="rId34" xr:uid="{E6536F8F-18BD-4BC3-89DE-07E2493DE473}"/>
+    <hyperlink ref="I36" r:id="rId35" xr:uid="{489AFC35-174F-4C73-8C99-B69B11CFD0D6}"/>
+    <hyperlink ref="I37" r:id="rId36" xr:uid="{991DB454-F8C9-4ED3-9D12-65EA2E5F46F9}"/>
+    <hyperlink ref="I38" r:id="rId37" xr:uid="{65CDA839-7D3F-42A3-A633-E39F470BA498}"/>
+    <hyperlink ref="I39" r:id="rId38" xr:uid="{E5747791-2A40-411D-9A01-BDE6E7584418}"/>
+    <hyperlink ref="I40" r:id="rId39" xr:uid="{A049187B-3088-45EE-88C1-534B500A917D}"/>
+    <hyperlink ref="I41" r:id="rId40" xr:uid="{747944F7-E8C7-4DF1-A70C-B7B35CBB6CDE}"/>
+    <hyperlink ref="I42" r:id="rId41" xr:uid="{ADF55A41-8B39-4CB9-9669-DAC67E589D80}"/>
+    <hyperlink ref="I43" r:id="rId42" xr:uid="{706CC92C-FAEB-427A-AF8C-611C34C9A458}"/>
+    <hyperlink ref="I44" r:id="rId43" xr:uid="{39425781-5800-4CEF-BA4E-F7DB72A9D3CE}"/>
+    <hyperlink ref="I45" r:id="rId44" xr:uid="{F5ACAF66-2602-4B2E-8CAA-22A1B2771EA5}"/>
+    <hyperlink ref="I46" r:id="rId45" xr:uid="{2CF68D26-FD42-426A-8DF5-23012C7897AF}"/>
+    <hyperlink ref="I47" r:id="rId46" xr:uid="{7011A6B6-2084-4F7D-A238-43A4C7553609}"/>
+    <hyperlink ref="I48" r:id="rId47" xr:uid="{0B0111AD-7610-40BD-AC99-8E2A7E767019}"/>
+    <hyperlink ref="I49" r:id="rId48" xr:uid="{6D935D54-0709-413E-A935-7F694B725D1B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>